<commit_message>
puc goes agaisnt both sewer and taxes
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -114,7 +114,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\-yy"/>
     <numFmt numFmtId="165" formatCode="m/d/yy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="12.0"/>
       <color theme="1"/>
@@ -161,6 +161,12 @@
       <sz val="12.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12.0"/>
@@ -477,7 +483,7 @@
     <xf borderId="7" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="8" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -490,13 +496,13 @@
     <xf borderId="14" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="15" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="16" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="17" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -729,7 +735,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="24.33"/>
+    <col customWidth="1" min="1" max="1" width="28.89"/>
     <col customWidth="1" min="2" max="2" width="21.89"/>
     <col customWidth="1" min="3" max="4" width="14.67"/>
     <col customWidth="1" min="5" max="8" width="10.67"/>

</xml_diff>